<commit_message>
tested some correlations between flows and floods over time and tried plotting these data
</commit_message>
<xml_diff>
--- a/raw/Wetland_vege_components_summaries.xlsx
+++ b/raw/Wetland_vege_components_summaries.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unsw-my.sharepoint.com/personal/z5204897_ad_unsw_edu_au1/Documents/Desktop/Honours_UNSW/Assessment/cumbung_assessment/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="935" documentId="8_{DA5EBC64-D6EE-4587-932F-E39763AA9FB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DFEF8D44-5E85-44A4-9F5C-214634F07559}"/>
+  <xr:revisionPtr revIDLastSave="936" documentId="8_{DA5EBC64-D6EE-4587-932F-E39763AA9FB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F303C3EE-B84B-4886-A6AC-3B89D0BD312E}"/>
   <bookViews>
-    <workbookView xWindow="12" yWindow="12" windowWidth="10692" windowHeight="13536" firstSheet="1" activeTab="4" xr2:uid="{9F335763-5C09-48D9-8601-B6DFE4C07C30}"/>
+    <workbookView xWindow="12" yWindow="12" windowWidth="22968" windowHeight="12384" firstSheet="1" activeTab="3" xr2:uid="{9F335763-5C09-48D9-8601-B6DFE4C07C30}"/>
   </bookViews>
   <sheets>
     <sheet name="All_ANAE" sheetId="6" r:id="rId1"/>
@@ -8890,6 +8890,10 @@
       <c r="K15" s="3" t="s">
         <v>58</v>
       </c>
+      <c r="N15">
+        <f>N14/SUM(N14:W14)</f>
+        <v>4.1751527494908347E-2</v>
+      </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
@@ -11386,7 +11390,7 @@
         <v>5.4812704313943823E-4</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A83" s="1" t="s">
         <v>134</v>
       </c>
@@ -11415,7 +11419,7 @@
         <v>1.2927565000352713E-2</v>
       </c>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A84" s="1" t="s">
         <v>136</v>
       </c>
@@ -11444,7 +11448,7 @@
         <v>2.26345886160001E-3</v>
       </c>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A85" s="1" t="s">
         <v>144</v>
       </c>
@@ -11502,7 +11506,7 @@
         <v>1.5829074423562257E-5</v>
       </c>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A87" s="1" t="s">
         <v>135</v>
       </c>
@@ -11531,7 +11535,7 @@
         <v>6.3377026202546732E-6</v>
       </c>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A88" s="1" t="s">
         <v>65</v>
       </c>
@@ -11589,7 +11593,7 @@
         <v>1.3829218029234551E-2</v>
       </c>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A90" s="1" t="s">
         <v>67</v>
       </c>
@@ -11618,7 +11622,7 @@
         <v>4.7538223495471495E-2</v>
       </c>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A91" s="1" t="s">
         <v>68</v>
       </c>
@@ -11705,7 +11709,7 @@
         <v>0.60734645859993752</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A94" s="1" t="s">
         <v>71</v>
       </c>
@@ -11734,7 +11738,7 @@
         <v>6.5974246027192991E-3</v>
       </c>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A95" s="1" t="s">
         <v>72</v>
       </c>
@@ -11821,7 +11825,7 @@
         <v>1.5363023009061913E-3</v>
       </c>
     </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A98" s="1" t="s">
         <v>75</v>
       </c>
@@ -11850,7 +11854,7 @@
         <v>7.1568062044263664E-3</v>
       </c>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A99" s="1" t="s">
         <v>76</v>
       </c>
@@ -11879,7 +11883,7 @@
         <v>4.2710064656564847E-5</v>
       </c>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A100" s="1" t="s">
         <v>77</v>
       </c>
@@ -11937,7 +11941,7 @@
         <v>2.1025109531327374E-3</v>
       </c>
     </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A102" s="1" t="s">
         <v>79</v>
       </c>
@@ -11966,7 +11970,7 @@
         <v>0.13456734440892645</v>
       </c>
     </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A103" s="1" t="s">
         <v>80</v>
       </c>
@@ -12024,7 +12028,7 @@
         <v>2.1738710905923934E-2</v>
       </c>
     </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A105" s="1" t="s">
         <v>82</v>
       </c>
@@ -12053,7 +12057,7 @@
         <v>2.3187671809450149E-5</v>
       </c>
     </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A106" s="1" t="s">
         <v>83</v>
       </c>
@@ -12082,7 +12086,7 @@
         <v>2.6764977620971854E-5</v>
       </c>
     </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A107" s="1" t="s">
         <v>84</v>
       </c>
@@ -12111,7 +12115,7 @@
         <v>1.7241579846707426E-5</v>
       </c>
     </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A108" s="1" t="s">
         <v>85</v>
       </c>
@@ -12169,7 +12173,7 @@
         <v>3.064816413842324E-4</v>
       </c>
     </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A110" s="1" t="s">
         <v>87</v>
       </c>
@@ -12198,7 +12202,7 @@
         <v>3.8170877483025662E-4</v>
       </c>
     </row>
-    <row r="111" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A111" s="1" t="s">
         <v>88</v>
       </c>
@@ -12227,7 +12231,7 @@
         <v>3.8253219719376112E-7</v>
       </c>
     </row>
-    <row r="112" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A112" s="1" t="s">
         <v>89</v>
       </c>
@@ -12256,7 +12260,7 @@
         <v>1.8434921799629561E-5</v>
       </c>
     </row>
-    <row r="113" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A113" s="1" t="s">
         <v>90</v>
       </c>
@@ -12285,7 +12289,7 @@
         <v>3.2115417115858462E-2</v>
       </c>
     </row>
-    <row r="114" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A114" s="1" t="s">
         <v>91</v>
       </c>
@@ -12314,7 +12318,7 @@
         <v>2.1641947182530016E-6</v>
       </c>
     </row>
-    <row r="115" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A115" s="1" t="s">
         <v>92</v>
       </c>
@@ -12343,7 +12347,7 @@
         <v>1.5147424304005881E-3</v>
       </c>
     </row>
-    <row r="116" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A116" s="1" t="s">
         <v>93</v>
       </c>
@@ -12401,7 +12405,7 @@
         <v>2.3407054720014793E-7</v>
       </c>
     </row>
-    <row r="118" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A118" s="1" t="s">
         <v>113</v>
       </c>
@@ -12430,7 +12434,7 @@
         <v>5.8125115362798588E-5</v>
       </c>
     </row>
-    <row r="119" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A119" s="1" t="s">
         <v>114</v>
       </c>
@@ -12720,7 +12724,7 @@
         <v>5.5435914105402394E-3</v>
       </c>
     </row>
-    <row r="129" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A129" s="1" t="s">
         <v>121</v>
       </c>
@@ -12778,7 +12782,7 @@
         <v>0.10742020999675939</v>
       </c>
     </row>
-    <row r="131" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A131" s="1" t="s">
         <v>125</v>
       </c>
@@ -12807,7 +12811,7 @@
         <v>7.1477944959629053E-5</v>
       </c>
     </row>
-    <row r="132" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A132" s="1" t="s">
         <v>135</v>
       </c>
@@ -12865,7 +12869,7 @@
         <v>1.7623726212716455E-4</v>
       </c>
     </row>
-    <row r="134" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A134" s="1" t="s">
         <v>121</v>
       </c>
@@ -12894,7 +12898,7 @@
         <v>0.1022208676986003</v>
       </c>
     </row>
-    <row r="135" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A135" s="1" t="s">
         <v>123</v>
       </c>
@@ -12952,7 +12956,7 @@
         <v>0.1170554074868127</v>
       </c>
     </row>
-    <row r="137" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A137" s="1" t="s">
         <v>132</v>
       </c>
@@ -12981,7 +12985,7 @@
         <v>1.0632275397995841E-2</v>
       </c>
     </row>
-    <row r="138" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A138" s="1" t="s">
         <v>120</v>
       </c>
@@ -13039,7 +13043,7 @@
         <v>9.7828993283857316E-2</v>
       </c>
     </row>
-    <row r="140" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A140" s="1" t="s">
         <v>124</v>
       </c>
@@ -13068,7 +13072,7 @@
         <v>3.912536368888192E-2</v>
       </c>
     </row>
-    <row r="141" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A141" s="1" t="s">
         <v>125</v>
       </c>
@@ -13097,7 +13101,7 @@
         <v>0.11110319286893579</v>
       </c>
     </row>
-    <row r="142" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A142" s="1" t="s">
         <v>127</v>
       </c>
@@ -13126,7 +13130,7 @@
         <v>3.51380594215011E-5</v>
       </c>
     </row>
-    <row r="143" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A143" s="1" t="s">
         <v>101</v>
       </c>
@@ -13155,7 +13159,7 @@
         <v>6.2503872941554635E-3</v>
       </c>
     </row>
-    <row r="144" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A144" s="1" t="s">
         <v>128</v>
       </c>
@@ -13184,7 +13188,7 @@
         <v>4.9528060247809296E-3</v>
       </c>
     </row>
-    <row r="145" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A145" s="1" t="s">
         <v>126</v>
       </c>
@@ -13213,7 +13217,7 @@
         <v>9.7426785675094E-3</v>
       </c>
     </row>
-    <row r="146" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A146" s="1" t="s">
         <v>144</v>
       </c>
@@ -13300,7 +13304,7 @@
         <v>0.13644907289896979</v>
       </c>
     </row>
-    <row r="149" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A149" s="1" t="s">
         <v>76</v>
       </c>
@@ -13329,7 +13333,7 @@
         <v>8.1846403934512368E-3</v>
       </c>
     </row>
-    <row r="150" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A150" s="1" t="s">
         <v>85</v>
       </c>
@@ -13358,7 +13362,7 @@
         <v>1.7523763920937672E-4</v>
       </c>
     </row>
-    <row r="151" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A151" s="1" t="s">
         <v>150</v>
       </c>
@@ -13387,7 +13391,7 @@
         <v>3.2617010389821739E-2</v>
       </c>
     </row>
-    <row r="152" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A152" s="1" t="s">
         <v>151</v>
       </c>
@@ -13416,7 +13420,7 @@
         <v>7.761179467420673E-2</v>
       </c>
     </row>
-    <row r="153" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A153" s="1" t="s">
         <v>119</v>
       </c>
@@ -13503,7 +13507,7 @@
         <v>1.3072545991570607E-2</v>
       </c>
     </row>
-    <row r="156" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A156" s="1" t="s">
         <v>154</v>
       </c>
@@ -13532,7 +13536,7 @@
         <v>8.619391748157278E-3</v>
       </c>
     </row>
-    <row r="157" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A157" s="1" t="s">
         <v>136</v>
       </c>
@@ -13561,7 +13565,7 @@
         <v>1.7428283490469834E-2</v>
       </c>
     </row>
-    <row r="158" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A158" s="1" t="s">
         <v>155</v>
       </c>
@@ -13619,7 +13623,7 @@
         <v>1.5832932195874847E-4</v>
       </c>
     </row>
-    <row r="160" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A160" s="1" t="s">
         <v>100</v>
       </c>
@@ -13677,7 +13681,7 @@
         <v>4.1884643594716289E-2</v>
       </c>
     </row>
-    <row r="162" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A162" s="1" t="s">
         <v>130</v>
       </c>
@@ -13706,7 +13710,7 @@
         <v>3.2720736258678293E-3</v>
       </c>
     </row>
-    <row r="163" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A163" s="1" t="s">
         <v>157</v>
       </c>
@@ -13735,7 +13739,7 @@
         <v>1.3745334493014455E-3</v>
       </c>
     </row>
-    <row r="164" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A164" s="1" t="s">
         <v>137</v>
       </c>
@@ -13764,7 +13768,7 @@
         <v>2.2851756870725142E-2</v>
       </c>
     </row>
-    <row r="165" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A165" s="1" t="s">
         <v>158</v>
       </c>
@@ -13793,7 +13797,7 @@
         <v>4.797288291566304E-5</v>
       </c>
     </row>
-    <row r="166" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A166" s="1" t="s">
         <v>159</v>
       </c>
@@ -13822,7 +13826,7 @@
         <v>1.8720940256044546E-5</v>
       </c>
     </row>
-    <row r="167" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A167" s="1" t="s">
         <v>160</v>
       </c>
@@ -13851,7 +13855,7 @@
         <v>9.5461262221075587E-4</v>
       </c>
     </row>
-    <row r="168" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A168" s="1" t="s">
         <v>142</v>
       </c>
@@ -13909,7 +13913,7 @@
         <v>3.1440431065571134E-5</v>
       </c>
     </row>
-    <row r="170" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A170" s="1" t="s">
         <v>138</v>
       </c>
@@ -13938,7 +13942,7 @@
         <v>7.7236672750943377E-5</v>
       </c>
     </row>
-    <row r="171" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A171" s="1" t="s">
         <v>161</v>
       </c>
@@ -13967,7 +13971,7 @@
         <v>2.8932837976569614E-7</v>
       </c>
     </row>
-    <row r="172" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A172" s="1" t="s">
         <v>162</v>
       </c>
@@ -13996,7 +14000,7 @@
         <v>9.3298197124464145E-5</v>
       </c>
     </row>
-    <row r="173" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A173" s="1" t="s">
         <v>84</v>
       </c>
@@ -14083,7 +14087,7 @@
         <v>1.082215230519128E-2</v>
       </c>
     </row>
-    <row r="176" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A176" s="1" t="s">
         <v>65</v>
       </c>
@@ -14112,7 +14116,7 @@
         <v>3.0359468588599434E-2</v>
       </c>
     </row>
-    <row r="177" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A177" s="1" t="s">
         <v>90</v>
       </c>
@@ -14141,7 +14145,7 @@
         <v>0.13640855327273657</v>
       </c>
     </row>
-    <row r="178" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A178" s="1" t="s">
         <v>67</v>
       </c>
@@ -14170,7 +14174,7 @@
         <v>3.5216204652854837E-4</v>
       </c>
     </row>
-    <row r="179" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A179" s="1" t="s">
         <v>80</v>
       </c>
@@ -14257,7 +14261,7 @@
         <v>4.3496092863693717E-3</v>
       </c>
     </row>
-    <row r="182" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A182" s="1" t="s">
         <v>72</v>
       </c>
@@ -14373,7 +14377,7 @@
         <v>5.5378544603500904E-2</v>
       </c>
     </row>
-    <row r="186" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A186" s="1" t="s">
         <v>93</v>
       </c>
@@ -14402,7 +14406,7 @@
         <v>7.6175776347291405E-2</v>
       </c>
     </row>
-    <row r="187" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A187" s="1" t="s">
         <v>75</v>
       </c>
@@ -14431,7 +14435,7 @@
         <v>6.1287220036521251E-3</v>
       </c>
     </row>
-    <row r="188" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A188" s="1" t="s">
         <v>96</v>
       </c>
@@ -14489,7 +14493,7 @@
         <v>8.2082638002227828E-2</v>
       </c>
     </row>
-    <row r="190" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A190" s="1" t="s">
         <v>98</v>
       </c>
@@ -14547,7 +14551,7 @@
         <v>1.1641513478186287E-3</v>
       </c>
     </row>
-    <row r="192" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A192" s="1" t="s">
         <v>71</v>
       </c>
@@ -14576,7 +14580,7 @@
         <v>5.4346393622855156E-3</v>
       </c>
     </row>
-    <row r="193" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A193" s="1" t="s">
         <v>91</v>
       </c>
@@ -14634,7 +14638,7 @@
         <v>5.0086921880796286E-3</v>
       </c>
     </row>
-    <row r="195" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A195" s="1" t="s">
         <v>100</v>
       </c>
@@ -14692,7 +14696,7 @@
         <v>3.8859963999338873E-2</v>
       </c>
     </row>
-    <row r="197" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A197" s="1" t="s">
         <v>101</v>
       </c>
@@ -14750,7 +14754,7 @@
         <v>1.397599126842493E-2</v>
       </c>
     </row>
-    <row r="199" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A199" s="1" t="s">
         <v>102</v>
       </c>
@@ -14837,7 +14841,7 @@
         <v>1.3355791378869612E-2</v>
       </c>
     </row>
-    <row r="202" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A202" s="1" t="s">
         <v>104</v>
       </c>
@@ -14895,7 +14899,7 @@
         <v>5.5311241167148506E-3</v>
       </c>
     </row>
-    <row r="204" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A204" s="1" t="s">
         <v>106</v>
       </c>
@@ -14953,7 +14957,7 @@
         <v>1.5958553720492793E-5</v>
       </c>
     </row>
-    <row r="206" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A206" s="1" t="s">
         <v>108</v>
       </c>
@@ -14982,7 +14986,7 @@
         <v>1.5631626455648959E-3</v>
       </c>
     </row>
-    <row r="207" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A207" s="1" t="s">
         <v>109</v>
       </c>
@@ -15011,7 +15015,7 @@
         <v>2.9933807354111814E-5</v>
       </c>
     </row>
-    <row r="208" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A208" s="1" t="s">
         <v>110</v>
       </c>
@@ -15040,7 +15044,7 @@
         <v>9.1051754406672389E-3</v>
       </c>
     </row>
-    <row r="209" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A209" s="1" t="s">
         <v>84</v>
       </c>
@@ -15069,7 +15073,7 @@
         <v>8.9201271558753681E-3</v>
       </c>
     </row>
-    <row r="210" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A210" s="1" t="s">
         <v>85</v>
       </c>
@@ -15098,7 +15102,7 @@
         <v>7.6899040261974808E-4</v>
       </c>
     </row>
-    <row r="211" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A211" s="1" t="s">
         <v>111</v>
       </c>
@@ -15127,7 +15131,7 @@
         <v>2.6445145527056176E-2</v>
       </c>
     </row>
-    <row r="212" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A212" s="1" t="s">
         <v>112</v>
       </c>
@@ -15156,7 +15160,7 @@
         <v>2.2902765496200638E-2</v>
       </c>
     </row>
-    <row r="213" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A213" s="1" t="s">
         <v>113</v>
       </c>
@@ -15185,7 +15189,7 @@
         <v>8.9460740183782902E-3</v>
       </c>
     </row>
-    <row r="214" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A214" s="1" t="s">
         <v>114</v>
       </c>
@@ -15214,7 +15218,7 @@
         <v>5.9225154172276445E-2</v>
       </c>
     </row>
-    <row r="215" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A215" s="1" t="s">
         <v>87</v>
       </c>
@@ -15243,7 +15247,7 @@
         <v>5.9291695499654598E-5</v>
       </c>
     </row>
-    <row r="216" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A216" s="1" t="s">
         <v>115</v>
       </c>
@@ -15272,7 +15276,7 @@
         <v>2.7615341299266555E-6</v>
       </c>
     </row>
-    <row r="217" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A217" s="1" t="s">
         <v>116</v>
       </c>
@@ -15301,7 +15305,7 @@
         <v>1.4912659214373061E-4</v>
       </c>
     </row>
-    <row r="218" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A218" s="1" t="s">
         <v>117</v>
       </c>
@@ -15330,7 +15334,7 @@
         <v>8.9922053617747636E-5</v>
       </c>
     </row>
-    <row r="219" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A219" s="1" t="s">
         <v>118</v>
       </c>
@@ -15359,7 +15363,7 @@
         <v>3.2018035884122957E-6</v>
       </c>
     </row>
-    <row r="220" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A220" s="1" t="s">
         <v>83</v>
       </c>
@@ -15417,7 +15421,7 @@
         <v>1.2025228204983853E-3</v>
       </c>
     </row>
-    <row r="222" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A222" s="1" t="s">
         <v>141</v>
       </c>
@@ -15446,7 +15450,7 @@
         <v>1.3230516101435253E-5</v>
       </c>
     </row>
-    <row r="223" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A223" s="1" t="s">
         <v>127</v>
       </c>
@@ -15504,7 +15508,7 @@
         <v>0.21040275647286136</v>
       </c>
     </row>
-    <row r="225" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A225" s="1" t="s">
         <v>65</v>
       </c>
@@ -15533,7 +15537,7 @@
         <v>1.9970378641982579E-2</v>
       </c>
     </row>
-    <row r="226" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A226" s="1" t="s">
         <v>174</v>
       </c>
@@ -15562,7 +15566,7 @@
         <v>9.9075803427406794E-2</v>
       </c>
     </row>
-    <row r="227" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A227" s="1" t="s">
         <v>113</v>
       </c>
@@ -15591,7 +15595,7 @@
         <v>1.7680379756762791E-2</v>
       </c>
     </row>
-    <row r="228" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A228" s="1" t="s">
         <v>114</v>
       </c>
@@ -15620,7 +15624,7 @@
         <v>5.3542635400697126E-3</v>
       </c>
     </row>
-    <row r="229" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A229" s="1" t="s">
         <v>175</v>
       </c>
@@ -15649,7 +15653,7 @@
         <v>1.606329731624299E-3</v>
       </c>
     </row>
-    <row r="230" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A230" s="1" t="s">
         <v>108</v>
       </c>
@@ -15734,7 +15738,7 @@
         <v>1.2353736025239087E-3</v>
       </c>
     </row>
-    <row r="233" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A233" s="1" t="s">
         <v>127</v>
       </c>
@@ -15792,7 +15796,7 @@
         <v>1.0306227559648017E-2</v>
       </c>
     </row>
-    <row r="235" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A235" s="1" t="s">
         <v>65</v>
       </c>
@@ -15821,7 +15825,7 @@
         <v>3.1361150661174161E-2</v>
       </c>
     </row>
-    <row r="236" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A236" s="1" t="s">
         <v>90</v>
       </c>
@@ -15850,7 +15854,7 @@
         <v>1.3324271150473368E-4</v>
       </c>
     </row>
-    <row r="237" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A237" s="1" t="s">
         <v>174</v>
       </c>
@@ -15879,7 +15883,7 @@
         <v>6.2241242394066192E-2</v>
       </c>
     </row>
-    <row r="238" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A238" s="1" t="s">
         <v>113</v>
       </c>
@@ -15908,7 +15912,7 @@
         <v>0.87106449468615055</v>
       </c>
     </row>
-    <row r="239" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A239" s="1" t="s">
         <v>114</v>
       </c>
@@ -15937,7 +15941,7 @@
         <v>1.670293225847564E-2</v>
       </c>
     </row>
-    <row r="240" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A240" s="1" t="s">
         <v>175</v>
       </c>
@@ -15966,7 +15970,7 @@
         <v>3.6245967325156624E-5</v>
       </c>
     </row>
-    <row r="241" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A241" s="1" t="s">
         <v>108</v>
       </c>

</xml_diff>